<commit_message>
Añadir columna 'Notas' para anotaciones del archivero e integrar en sincronizador Excel/CSV
</commit_message>
<xml_diff>
--- a/Nivel 9 (Documento simple).xlsx
+++ b/Nivel 9 (Documento simple).xlsx
@@ -10,7 +10,7 @@
     <sheet name="Nivel 9 (Documento simple)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nivel 9 (Documento simple)'!$A$1:$L$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nivel 9 (Documento simple)'!$A$1:$M$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L9"/>
+  <dimension ref="A1:M9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -469,6 +469,7 @@
     <col width="35" customWidth="1" min="10" max="10"/>
     <col width="30" customWidth="1" min="11" max="11"/>
     <col width="45" customWidth="1" min="12" max="12"/>
+    <col width="40" customWidth="1" min="13" max="13"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
@@ -532,6 +533,11 @@
           <t>subject</t>
         </is>
       </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
     </row>
     <row r="2" ht="22" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
@@ -594,6 +600,7 @@
           <t>Guerra Civil Española, Atarazanas, Recortables, Memoria histórica, Ilustraciones</t>
         </is>
       </c>
+      <c r="M2" s="3" t="inlineStr"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
@@ -652,6 +659,7 @@
           <t>Columna Durruti, Milicias del Pueblo, CNT-FAI, Anarquismo, Propaganda de guerra</t>
         </is>
       </c>
+      <c r="M3" s="3" t="inlineStr"/>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
@@ -706,6 +714,11 @@
           <t>El Refractor, Sellos de caucho, Imprenta, Movimiento libertario, Objetos</t>
         </is>
       </c>
+      <c r="M4" s="3" t="inlineStr">
+        <is>
+          <t>Ubicacion física no definitiva</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
@@ -764,6 +777,11 @@
           <t>Sindicato Único, Industrias Químicas, CNT-AIT, Colectivizaciones, Cerillas</t>
         </is>
       </c>
+      <c r="M5" s="3" t="inlineStr">
+        <is>
+          <t>Ubicacion física no definitiva</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
@@ -826,6 +844,11 @@
           <t>Anarquismo individualista, Émile Armand, Pepitas de Calabaza, Libros, Ex-libris</t>
         </is>
       </c>
+      <c r="M6" s="3" t="inlineStr">
+        <is>
+          <t>Ubicacion física no definitiva</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
@@ -880,6 +903,11 @@
           <t>Abstencionismo, Casas Viejas, Segunda República, Pasquines, Propaganda</t>
         </is>
       </c>
+      <c r="M7" s="3" t="inlineStr">
+        <is>
+          <t>Ubicacion física no definitiva</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
@@ -938,6 +966,11 @@
           <t>José Díaz, Partido Comunista de España, Banderines, Simbología política, Guerra Civil Española</t>
         </is>
       </c>
+      <c r="M8" s="3" t="inlineStr">
+        <is>
+          <t>Ubicacion física no definitiva</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
@@ -996,9 +1029,14 @@
           <t>Servicio de Investigación Militar, Banderas, Segunda República, Guiones militares, Guerra Civil Española</t>
         </is>
       </c>
+      <c r="M9" s="3" t="inlineStr">
+        <is>
+          <t>Ubicacion física no definitiva</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L9"/>
+  <autoFilter ref="A1:M9"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Catalogación de documentos D004 a D048, actualización de CSV/Excel y optimizaciones del buscador UI
</commit_message>
<xml_diff>
--- a/Nivel 9 (Documento simple).xlsx
+++ b/Nivel 9 (Documento simple).xlsx
@@ -10,7 +10,7 @@
     <sheet name="Nivel 9 (Documento simple)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nivel 9 (Documento simple)'!$A$1:$M$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nivel 9 (Documento simple)'!$A$1:$M$49</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M9"/>
+  <dimension ref="A1:M49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -723,12 +723,12 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D004.jpg</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D004.jpg</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D004</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D004</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
@@ -753,7 +753,7 @@
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>MILITANCIA</t>
+          <t>PUBLICACIONES</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1035,8 +1035,2352 @@
         </is>
       </c>
     </row>
+    <row r="10" ht="22" customHeight="1">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C002-P003-D009.jpg</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C002-P003-D009</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>C002-P003</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>[Correo electrónico de Koldo Artieda a Rafael Zarza sobre Alfonso Laurencic y las chekas de Barcelona]</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Correo electrónico impreso remitido por Koldo Artieda a Rafael Zarza solicitando información sobre el arquitecto y diseñador Alfonso Laurencic y la construcción de las chekas decorativas en Barcelona durante la Guerra Civil Española.</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>2010-05-27</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>Impresión sobre papel</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>Koldo Artieda</t>
+        </is>
+      </c>
+      <c r="L10" s="3" t="inlineStr">
+        <is>
+          <t>Alfonso Laurencic, Chekas, Guerra Civil Española, Correspondencia</t>
+        </is>
+      </c>
+      <c r="M10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="22" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C004-P003-D010.jpg</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C004-P003-D010</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>C004-P003</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>CO.IN comunicado nº 2 .... ¡¡A GRAZALEMA!!! es el LEMA...</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Comunicado manuscrito a 2 folios de CO.IN (Coordinadora Insurrecta) firmado por ZRZ el 7 de julio de 2008 (día de San Fermín) proponiendo una concentración y exposición en Grazalema sobre el legado y cenizas de Quico Rivas ("Q.R."), incluyendo lemas como "HONOR A Q.R" y "QUICO ES NUESTRO!".</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>2008-07-07</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>Grazalema</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>Manuscrito a bolígrafo sobre papel (2 folios)</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>Eva Rivas, ZRZ, Quico Rivas, Alejandro RajKuter</t>
+        </is>
+      </c>
+      <c r="L11" s="3" t="inlineStr">
+        <is>
+          <t>CO.IN, Quico Rivas, Grazalema, Comunicados, Manuscritos</t>
+        </is>
+      </c>
+      <c r="M11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12" ht="22" customHeight="1">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C006-P001-D011.jpg</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C006-P001-D011</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>C006-P001</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>[Nota manuscrita sobre la custodia de la documentación del Archivo Refractor]</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Nota manuscrita a lápiz por D-RajKuter formalizando la entrega y custodia temporal a Rafael Zarza de la documentación del Archivo Refractor para su digitalización y depósito final en la Fundación CEDCS.</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>Manuscrito a lápiz sobre papel</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>D-RajKuter</t>
+        </is>
+      </c>
+      <c r="L12" s="3" t="inlineStr">
+        <is>
+          <t>El Refractor, Archivo Refractor, CEDCS, Custodia de documentos</t>
+        </is>
+      </c>
+      <c r="M12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="22" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C006-P001-D012.jpg</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C006-P001-D012</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>C006-P001</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>[Boceto gráfico con silueta dentada circular sobre fondo morado]</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Composición gráfica original realizada en gouache y tinta compuesta por una figura circular dentada negra sobre un panel de fondo morado violáceo.</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr"/>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>Gouache y tinta sobre papel</t>
+        </is>
+      </c>
+      <c r="K13" s="3" t="inlineStr"/>
+      <c r="L13" s="3" t="inlineStr">
+        <is>
+          <t>Bocetos, Diseño gráfico, Contracultura, Obra gráfica</t>
+        </is>
+      </c>
+      <c r="M13" s="3" t="inlineStr"/>
+    </row>
+    <row r="14" ht="22" customHeight="1">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C006-P001-D013.jpg</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C006-P001-D013</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>C006-P001</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de viaje a la URSS de Daniel Zarza y caligrafía de texto de Alejandro Rossi]</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Composición combinada con tarjeta desplegable de la URSS enviada por Daniel Zarza en 1983 y caligrafía artística a tinta de una reflexión literaria sobre la pintura atribuida a Alejandro Rossi.</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>1983</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAL</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>Collage, tinta y tarjeta postal sobre papel</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>Daniel Zarza, Alejandro Rossi</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Daniel Zarza, URSS, Alejandro Rossi, Caligrafía, Tarjetas postales</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="22" customHeight="1">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C006-P001-D014.jpg</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C006-P001-D014</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>C006-P001</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Pintura suprematista 1916</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Rafael Zarza firmado bajo el monograma Z®Z, compuesto por dibujo a tinta y gouache de utensilios de estudio (vaso con pinceles, caja de pasteles, lápiz y goma) e inserción recortada de una composición de pintura suprematista de Kazimir Malevich de 1916.</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAL</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr"/>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>Collage, tinta y gouache sobre papel</t>
+        </is>
+      </c>
+      <c r="K15" s="3" t="inlineStr"/>
+      <c r="L15" s="3" t="inlineStr">
+        <is>
+          <t>Kazimir Malevich, Suprematismo, Collage, Zarza, Z®Z</t>
+        </is>
+      </c>
+      <c r="M15" s="3" t="inlineStr"/>
+    </row>
+    <row r="16" ht="22" customHeight="1">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C006-P001-D015.jpg</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C006-P001-D015</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>C006-P001</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Autorretrato 1933</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Rafael Zarza firmado bajo el monograma Z®Z en el ángulo inferior derecho, compuesto por dibujo a tinta de utensilios de estudio e inserción recortada del Autorretrato de Kazimir Malevich de 1933.</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAL</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>Collage, tinta y gouache sobre papel</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr"/>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Kazimir Malevich, Suprematismo, Collage, Zarza, Z®Z</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="22" customHeight="1">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C006-P002-D016.jpg</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C006-P002-D016</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>C006-P002</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>DOMINGO NEGRO 31-V-98. EL ESTADO ES LA OBRA DE ARTE. DEMOLICIÓN 4</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Cartel impreso del evento "Domingo Negro" (31-V-98) organizado conjuntamente por El Ojo Atómico y El Refractor en C/ Bocángel 59, Madrid. Incluye ilustración firmada por C. El Fiera, corrección manuscrita ("esta mal") en la hora y la programación completa con Javier Pérez Aranda, Josechu Davila, G.R.R.R. (T), Rag Cutter y Manolo La UVI.</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>1998-05-31</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>Madrid, Calle Bocángel 59</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>Cartel impreso sobre papel</t>
+        </is>
+      </c>
+      <c r="K17" s="3" t="inlineStr">
+        <is>
+          <t>El Ojo Atómico, El Refractor, C. El Fiera, Javier Pérez Aranda, Josechu Davila, G.R.R.R. (T), Rag Cutter, Manolo La UVI</t>
+        </is>
+      </c>
+      <c r="L17" s="3" t="inlineStr">
+        <is>
+          <t>El Ojo Atómico, El Refractor, Domingo Negro, Bocángel 59, Carteles</t>
+        </is>
+      </c>
+      <c r="M17" s="3" t="inlineStr"/>
+    </row>
+    <row r="18" ht="22" customHeight="1">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C007-P001-D017.jpg</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C007-P001-D017</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>C007-P001</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>REFRACTOR, LA GEOMETRÍA Y LA MUERTE. Nota (Aclaración a una información de EL MUNDO)</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Manuscrito original de 4 folios firmado por Quico Rivas para el periódico El Refractor aclarando la polémica cobertura mediática en El Mundo sobre la instalación del colectivo mexicano SEMEFO en la galería Cruce.</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>1998-03-10</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>Manuscrito a bolígrafo sobre papel</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Grupo SEMEFO, Galería Cruce, Lorenzo Mandinga, KAX-1013</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>El Refractor, Quico Rivas, SEMEFO, Galería Cruce, ZAT, KAX-1013</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="22" customHeight="1">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C007-P002-D018.jpg</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C007-P002-D018</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>C007-P002</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía artística en blanco y negro de una puerta con pintadas anarquistas "DIOS ES NEGRA" y "ANARKIA P.G.B"]</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Tirada fotográfica artística en blanco y negro original firmada por Rafa Montesinos y numerada (7/25) retratando una puerta de entrada urbana con grafiti anarquista.</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>MILITANCIA</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K19" s="3" t="inlineStr">
+        <is>
+          <t>Rafa Montesinos</t>
+        </is>
+      </c>
+      <c r="L19" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía, Rafa Montesinos, Anarquismo, Grafitis</t>
+        </is>
+      </c>
+      <c r="M19" s="3" t="inlineStr"/>
+    </row>
+    <row r="20" ht="22" customHeight="1">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C007-P002-D019.jpg</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C007-P002-D019</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>C007-P002</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>MARAVILES 12-V-98. ¡NOS HAN CORTADO LA LUZ! LA BOLSA NEGRA ESTÁ VACÍA</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Comunicado manuscrito a rotulador sobre el corte de suministro del espacio Maraviles (C/ San Carlos 13) acompañado de una factura real de Iberdrola a nombre de Mblanca Sánchez Berciano / Skin Art.</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>1998-05-12</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>MILITANCIA</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>Manuscrito a rotulador sobre papel con factura adherida</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>Mblanca Sánchez Berciano, Skin Art</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Maraviles, Contracultura, Cortes de luz, Comunicados</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="22" customHeight="1">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C007-P002-D020.jpg</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C007-P002-D020</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>C007-P002</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>SEÑORES ANARQUISTAS: LOS CARTELES E INVITACIONES DE BOCANGEL ESTÁN FOTOCOPIÁNDOSE</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Nota manuscrita organizativa firmada por Willy dirigida al equipo/colectivo organizador de los eventos de Bocángel ("Señores Anarquistas"), comunicando la impresión de 30 carteles A3 (15 verdes y 15 amarillos) y 200 tarjetas por importe de 2.780 pesetas, solicitando que alguien acuda a recogerlos al local de fotocopias junto al Beirut.</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>Madrid, Calle Bocángel</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>Manuscrito a rotulador sobre papel</t>
+        </is>
+      </c>
+      <c r="K21" s="3" t="inlineStr">
+        <is>
+          <t>Willy, Quico Rivas, Mar</t>
+        </is>
+      </c>
+      <c r="L21" s="3" t="inlineStr">
+        <is>
+          <t>Bocángel, Carteles, Anarquismo, Imprenta, Notas manuscritas</t>
+        </is>
+      </c>
+      <c r="M21" s="3" t="inlineStr"/>
+    </row>
+    <row r="22" ht="22" customHeight="1">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D021.jpg</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D021</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>C025-P001</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>[Diorama recortable montado sobre cartón de la batalla de las Atarazanas de Barcelona]</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Diorama tridimensional montado sobre soporte rígido de cartón realizado a partir de la lámina recortable de la serie sobre la Guerra Civil en Barcelona (Atarazanas). Recrea la escena con árboles en primer plano y milicianos armados parapetados en la base.</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>Barcelona, Atarazanas</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Physical Object</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>Diorama tridimensional recortable montado sobre cartón</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>I. G. Offset</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Barcelona, Recortables, Guerra Civil Española, Atarazanas, Dioramas</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D022.jpg</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D022</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>C025-P001</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>[Collage alegórico con motivos de cine, teatro, pintura y artes gráficas]</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Collage original en blanco y negro de Rafael Zarza compuesto por recortes yuxtapuestos con celofán sobre papel blanco. Integra motivos alegóricos de las distintas disciplinas artísticas: bobina de cine, máscara teatral, figura humana con pluma y pincel y un ordenador personal.</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr"/>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>Collage de recortes fotomecánicos sobre papel</t>
+        </is>
+      </c>
+      <c r="K23" s="3" t="inlineStr"/>
+      <c r="L23" s="3" t="inlineStr">
+        <is>
+          <t>Collage, Rafael Zarza, Artes gráficas, Cine, Teatro</t>
+        </is>
+      </c>
+      <c r="M23" s="3" t="inlineStr"/>
+    </row>
+    <row r="24" ht="22" customHeight="1">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C025-P001-D023.jpg</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C025-P001-D023</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>C025-P001</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de diseño para el Sindicato de Industria del Espectáculo de la CNT-AIT]</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Rafael Zarza sobre soporte de cartulina roja que integra la composición gráfica alegórica del espectáculo junto con el texto tipográfico recortado "C.N.T. A.I.T. SINDICATO DE INDUSTRIA DEL ESPECTACULO" fijado en la parte inferior.</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>MILITANCIA</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>Collage de recortes fotomecánicos sobre cartulina roja</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>CNT-AIT Sindicato de Industria del Espectáculo</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>CNT-AIT, Sindicato del Espectáculo, Collage, Anarcosindicato, Diseño gráfico</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="22" customHeight="1">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D024.jpg</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D024</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>C025-P001</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>[Boceto de logotipo con pincel y bomba para Ediciones Refractarias: "No ahorréis pintura"]</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Estudio gráfico original de Rafael Zarza a tinta negra y roja sobre papel para el logotipo de Ediciones Refractarias. Muestra un pincel vertical acompañado del icono de una bomba y la leyenda dividida en bloques "NO AHORRÉIS PINTURA / EDICIONES / REFRACTARIAS".</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr"/>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="inlineStr">
+        <is>
+          <t>Dibujo a tinta sobre papel</t>
+        </is>
+      </c>
+      <c r="K25" s="3" t="inlineStr"/>
+      <c r="L25" s="3" t="inlineStr">
+        <is>
+          <t>Ediciones Refractarias, Bocetos, Diseños de logotipo, El Refractor, Rafael Zarza</t>
+        </is>
+      </c>
+      <c r="M25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D025.jpg</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D025</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>C025-P001</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>[Estudio de tipografía y composición para Ediciones Refractarias: "No ahorréis pintura"]</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Estudio de diseño original a tinta y collage de Rafael Zarza ensayando varias composiciones tipográficas y lemas manuscritos de "NO AHORRÉIS PINTURA" junto a dibujos de pincel y el pictograma del cuerpo humano con cabeza de bomba.</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>Tinta y collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr"/>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Ediciones Refractarias, Bocetos, Diseños de logotipo, El Refractor, Rafael Zarza</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="22" customHeight="1">
+      <c r="A27" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D026.jpg</t>
+        </is>
+      </c>
+      <c r="B27" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D026</t>
+        </is>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>C025-P001</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>[Diseño de dos emblemas circulares anarquistas para Ediciones Refractarias]</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Hoja de estudio gráfico original a tinta de Rafael Zarza con dos propuestas de logotipo circular para Ediciones Refractarias. Ambas composiciones reinterpretan la A circulada anarquista utilizando utensilios de artista (pinceles, compás y lápiz) rodeados por el texto periférico "NO AHORRÉIS PINTURA. EDICIONES REFRACTARIAS".</t>
+        </is>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H27" s="2" t="inlineStr"/>
+      <c r="I27" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J27" s="3" t="inlineStr">
+        <is>
+          <t>Tinta sobre papel</t>
+        </is>
+      </c>
+      <c r="K27" s="3" t="inlineStr"/>
+      <c r="L27" s="3" t="inlineStr">
+        <is>
+          <t>Ediciones Refractarias, Anarquismo, Logotipos, El Refractor, Rafael Zarza</t>
+        </is>
+      </c>
+      <c r="M27" s="3" t="inlineStr"/>
+    </row>
+    <row r="28" ht="22" customHeight="1">
+      <c r="A28" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D027.jpg</t>
+        </is>
+      </c>
+      <c r="B28" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C025-P001-D027</t>
+        </is>
+      </c>
+      <c r="C28" s="2" t="inlineStr">
+        <is>
+          <t>C025-P001</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>[Boceto en collage rojo y negro con la "A" para Ediciones Refractarias]</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Boceto y collage original de Rafael Zarza realizado en cartulina roja y tinta sobre papel desplegable. Representa una tipografía estilizada de la letra A anarquista construida a partir de lápices de dibujo, integrando los textos manuscritos "NO AHORRÉIS PINTURA" y "EDICIONES REFRACTARIAS".</t>
+        </is>
+      </c>
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Collage y tinta sobre papel desplegable</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr"/>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Ediciones Refractarias, Anarquismo, Logotipos, El Refractor, Rafael Zarza</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="22" customHeight="1">
+      <c r="A29" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C020-P002-D028.jpg</t>
+        </is>
+      </c>
+      <c r="B29" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C020-P002-D028</t>
+        </is>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>C020-P002</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>[Impresión sobre papel cebolla de una obra pictórica de Josechu Dávila]</t>
+        </is>
+      </c>
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>Reproducción impresa en blanco y negro sobre papel cebolla traslúcido de un cuadro del artista Josechu Dávila. Representa una estructura arquitectónica geométrica modulada en forma de celosía con entramado de sombras.</t>
+        </is>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H29" s="2" t="inlineStr"/>
+      <c r="I29" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J29" s="3" t="inlineStr">
+        <is>
+          <t>Impresión sobre papel cebolla traslúcido</t>
+        </is>
+      </c>
+      <c r="K29" s="3" t="inlineStr">
+        <is>
+          <t>Josechu Dávila</t>
+        </is>
+      </c>
+      <c r="L29" s="3" t="inlineStr">
+        <is>
+          <t>Josechu Dávila, Papel cebolla, Geometría, Obra pictórica</t>
+        </is>
+      </c>
+      <c r="M29" s="3" t="inlineStr"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="A30" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C024-P001-D029.jpg</t>
+        </is>
+      </c>
+      <c r="B30" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C024-P001-D029</t>
+        </is>
+      </c>
+      <c r="C30" s="2" t="inlineStr">
+        <is>
+          <t>C024-P001</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>DEL PANÓPTICO DE BENTHAM. LAS OTRAS GALERÍAS. AL PANÓPTICO DIGITAL</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>Collage de diseño original de Rafael Zarza compuesto como portada preparatoria para el proyecto de publicación "Las otras galerías". Presenta una composición de patrón geométrico óptico con la tipografía recortada del título principal flanqueada por los textos impresos "DEL PANÓPTICO DE BENTHAM" en la cabecera y "AL PANÓPTICO DIGITAL" en el pie.</t>
+        </is>
+      </c>
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H30" s="2" t="inlineStr"/>
+      <c r="I30" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>Collage de recortes fotomecánicos sobre papel</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr"/>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>Las otras galerías, Panóptico de Bentham, Panóptico digital, Design collage, Rafael Zarza</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D030.jpg</t>
+        </is>
+      </c>
+      <c r="B31" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D030</t>
+        </is>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D31" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con bola del mundo, lupa y etiqueta "GLASS STRAIGHT-SHANK"]</t>
+        </is>
+      </c>
+      <c r="E31" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas que combina un dibujo lineal a tinta de una esfera terrestre con recortes fotomecánicos de una lupa, la etiqueta comercial "GLASS STRAIGHT-SHANK Ø 75MM", una esfera lunar y elementos circulares. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H31" s="2" t="inlineStr"/>
+      <c r="I31" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J31" s="3" t="inlineStr">
+        <is>
+          <t>Collage y tinta sobre papel</t>
+        </is>
+      </c>
+      <c r="K31" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L31" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Esfera terrestre, Lupa, Los correctores</t>
+        </is>
+      </c>
+      <c r="M31" s="3" t="inlineStr"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="A32" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D031.jpg</t>
+        </is>
+      </c>
+      <c r="B32" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D031</t>
+        </is>
+      </c>
+      <c r="C32" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con militar socialista chino, automóvil descapotable rojo y retrato femenino con aparato facial]</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por un recorte de cartel de propaganda socialista china de un militar o guardia rojo, la fotografía de un automóvil descapotable clásico de color rojo (matrícula "BCH 100"), un sol y el retrato fotográfico en blanco y negro de una mujer portando un dispositivo facial metálico. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H32" s="2" t="inlineStr"/>
+      <c r="I32" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Propaganda china, Automóvil clásico, Los correctores</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33" ht="22" customHeight="1">
+      <c r="A33" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D032.jpg</t>
+        </is>
+      </c>
+      <c r="B33" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D032</t>
+        </is>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D33" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con silueta de cabeza, diagrama médico "Vasodilatación / Vasoconstricción" y prótesis dental]</t>
+        </is>
+      </c>
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas con trazo perfilado a tinta de una cabeza humana que alberga un esquema médico impreso sobre balanza ("Vasodilatación Antiproliferación Antitrómbico / Vasoconstricción Proliferación Protrombótico") con triángulo rosado central, y recortes inferiores de prótesis dental con puente odontológico. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H33" s="2" t="inlineStr"/>
+      <c r="I33" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J33" s="3" t="inlineStr">
+        <is>
+          <t>Collage y tinta sobre papel</t>
+        </is>
+      </c>
+      <c r="K33" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L33" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Anatomía, Odontología, Los correctores</t>
+        </is>
+      </c>
+      <c r="M33" s="3" t="inlineStr"/>
+    </row>
+    <row r="34" ht="22" customHeight="1">
+      <c r="A34" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D033.jpg</t>
+        </is>
+      </c>
+      <c r="B34" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D033</t>
+        </is>
+      </c>
+      <c r="C34" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con silueta de calavera con gafas de sol negras, nariz amarilla y dentadura con implante]</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas representando una cabeza/cráneo perfilada a tinta equipada con gafas de sol negras recortadas, una figura triangular de papel amarillo a modo de cavidad nasal y un recorte fotográfico de una dentadura con implante metálico. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H34" s="2" t="inlineStr"/>
+      <c r="I34" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>Collage y tinta sobre papel</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Calavera, Gafas de sol, Los correctores</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35" ht="22" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D034.jpg</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D034</t>
+        </is>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D35" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con automóvil azul Bugatti, articuladores odontológicos y cuadrados de color]</t>
+        </is>
+      </c>
+      <c r="E35" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por el recorte central de un deportivo azul Bugatti, dos fotografías impresas en blanco y negro de articuladores de moldes dentales y recortes de papeles de colores lisos (verde, rojo, azul jaspeado y retícula azul tipo gresite). Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H35" s="2" t="inlineStr"/>
+      <c r="I35" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J35" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K35" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L35" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Automóvil deportivo, Moldes dentales, Los correctores</t>
+        </is>
+      </c>
+      <c r="M35" s="3" t="inlineStr"/>
+    </row>
+    <row r="36" ht="22" customHeight="1">
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D035.jpg</t>
+        </is>
+      </c>
+      <c r="B36" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D035</t>
+        </is>
+      </c>
+      <c r="C36" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con diagrama vascular de aterosclerosis, flor anaranjada y retrato con arco facial]</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por un diagrama médico impreso sobre remodelado arterial ("Hipertensión / Dislipidemia / Aterosclerosis / RTP"), el recorte de una flor anaranjada entrelazada y el retrato fotográfico en blanco y negro de una mujer con arco facial odontológico. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H36" s="2" t="inlineStr"/>
+      <c r="I36" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Diagrama médico, Flor, Los correctores</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37" ht="22" customHeight="1">
+      <c r="A37" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D036.jpg</t>
+        </is>
+      </c>
+      <c r="B37" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D036</t>
+        </is>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D37" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con boca abierta, cápsula verde y amarilla y diagrama de cascada de caspasas]</t>
+        </is>
+      </c>
+      <c r="E37" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por la ilustración fotográfica de una boca abierta mostrando la cavidad bucal y campanilla sobre una cápsula farmacéutica verde y amarilla, y en la parte superior el diagrama de un proceso biológico celular ("Cascada de caspasas / Núcleo / Lesión"). Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H37" s="2" t="inlineStr"/>
+      <c r="I37" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J37" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K37" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L37" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Cápsula farmacéutica, Boca, Los correctores</t>
+        </is>
+      </c>
+      <c r="M37" s="3" t="inlineStr"/>
+    </row>
+    <row r="38" ht="22" customHeight="1">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D037.jpg</t>
+        </is>
+      </c>
+      <c r="B38" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D037</t>
+        </is>
+      </c>
+      <c r="C38" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con diagrama biofarmacéutico "Célula generadora / Célula diana", esquema de postura en silla y elemento gráfico negro]</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por un diagrama biofarmacéutico impreso sobre transferencia química celular ("CÉLULA GENERADORA / CÉLULA DIANA / GTP / GMPc / L-arginina / L-citrulina"), el recorte lineal de una persona sentada sobre una silla ergonómica de trabajo y un elemento gráfico en blanco y negro. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr"/>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Biofarmacia, Ergonomía, Los correctores</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39" ht="22" customHeight="1">
+      <c r="A39" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D038.jpg</t>
+        </is>
+      </c>
+      <c r="B39" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D038</t>
+        </is>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D39" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con tabla odontológica "Las cavidades de Columbia", instrumental quirúrgico y forma azul]</t>
+        </is>
+      </c>
+      <c r="E39" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por una tabla técnica impresa en blanco y negro con la clasificación de dentición "LAS CAVIDADES DE COLUMBIA DENTOFORM CORPORATION", el diagrama ergonómico de un cuerpo recostado, instrumental odontológico de exploración y una forma recortada de color azul. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H39" s="2" t="inlineStr"/>
+      <c r="I39" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J39" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K39" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L39" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Odontología, Instrumental médico, Los correctores</t>
+        </is>
+      </c>
+      <c r="M39" s="3" t="inlineStr"/>
+    </row>
+    <row r="40" ht="22" customHeight="1">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D039.jpg</t>
+        </is>
+      </c>
+      <c r="B40" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D039</t>
+        </is>
+      </c>
+      <c r="C40" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con elementos ensamblados en tótem, prótesis dental con perforaciones y paisaje marino]</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por una composición vertical a modo de tótem con recortes geométricos y mecánicos en blanco y negro, una plantilla de prótesis dental articulada con perforaciones y un recorte rectangular en la esquina inferior con textura de paisaje marino. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr"/>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Abstracción, Odontología, Los correctores</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41" ht="22" customHeight="1">
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D040.jpg</t>
+        </is>
+      </c>
+      <c r="B41" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D040</t>
+        </is>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D41" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con retratos masculinos, esquemas oculares y gafas de sol superpuestas]</t>
+        </is>
+      </c>
+      <c r="E41" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por tres retratos fotográficos recortados en blanco y negro del torso de un hombre en distintas posturas, acompañados de esquemas anatómicos impresos del sistema ocular y óptico, sobre los que se superponen recortes de tres modelos de gafas de sol. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H41" s="2" t="inlineStr"/>
+      <c r="I41" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J41" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K41" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L41" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Gafas de sol, Anatomía ocular, Los correctores</t>
+        </is>
+      </c>
+      <c r="M41" s="3" t="inlineStr"/>
+    </row>
+    <row r="42" ht="22" customHeight="1">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D041.jpg</t>
+        </is>
+      </c>
+      <c r="B42" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D041</t>
+        </is>
+      </c>
+      <c r="C42" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con miliciano chino, cuadro rojo, dibujo de mano con estilete y nota "Insuficiencia cardiaca refractaria"]</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por un recorte a color de propaganda socialista con la figura de un miliciano mirando al horizonte, un cuadrado de papel rojo intenso, el dibujo esquemático a tinta de una mano sujetando un estilete quirúrgico y un rótulo impreso con el texto "INSUFICIENCIA CARDIACA REFRACTARIA TRATAMIENTO MEDICO ECO: MALA FUNCION VENTRICULAR". Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr"/>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J42" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K42" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L42" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Propaganda china, Cardiología, Los correctores</t>
+        </is>
+      </c>
+      <c r="M42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43" ht="22" customHeight="1">
+      <c r="A43" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D042.jpg</t>
+        </is>
+      </c>
+      <c r="B43" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D042</t>
+        </is>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D43" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con mapa de Sevilla "SE-30", señal de conductor novel "L", calendario "Octubre 00" y tabla de puntos de accidentes]</t>
+        </is>
+      </c>
+      <c r="E43" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por un dibujo coloreado con la retícula urbana de Sevilla centrada en la autopista de circunvalación SE-30, un recorte de la señal oficial de conductor novel "L", un recorte rojo de calendario marcado "Octubre 00" y la tabla impresa "Zonas en las que se producen más accidentes en la ciudad" detallando 14 puntos viales (Puente V Centenario, Torneo, Ramón y Cajal, etc.). Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H43" s="2" t="inlineStr">
+        <is>
+          <t>Sevilla</t>
+        </is>
+      </c>
+      <c r="I43" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J43" s="3" t="inlineStr">
+        <is>
+          <t>Collage y cera sobre papel</t>
+        </is>
+      </c>
+      <c r="K43" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L43" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Sevilla, Tráfico, Los correctores</t>
+        </is>
+      </c>
+      <c r="M43" s="3" t="inlineStr"/>
+    </row>
+    <row r="44" ht="22" customHeight="1">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D043.jpg</t>
+        </is>
+      </c>
+      <c r="B44" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D043</t>
+        </is>
+      </c>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con milicianos socialistas chinos, gráfica farmacológica de Atenolol / Nebivolol y articulador de prótesis dental]</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por una ilustración de cartelería de propaganda socialista china con milicianos armados y campesinos en guardia, una gráfica estadística comparativa de fármacos ("ATENOLOL / NEBIVOLOL") y el recorte fotográfico en blanco y negro de un articulador de prótesis y moldes odontológicos. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr"/>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J44" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K44" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L44" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Propaganda china, Farmacología, Los correctores</t>
+        </is>
+      </c>
+      <c r="M44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45" ht="22" customHeight="1">
+      <c r="A45" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D044.jpg</t>
+        </is>
+      </c>
+      <c r="B45" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D044</t>
+        </is>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D45" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con miliciano chino, fotografía científica celular, cuadrado verde y gafas recortadas]</t>
+        </is>
+      </c>
+      <c r="E45" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por la ilustración de un miliciano socialista chino con uniforme verde y gorra con estrella roja ante un teléfono de baquelita, una fotografía científica en color de estructura celular/microscópica, un cuadrado de papel verde fosforito y un recorte de gafas de sol. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr"/>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J45" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K45" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L45" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Propaganda china, Micrografía, Los correctores</t>
+        </is>
+      </c>
+      <c r="M45" s="3" t="inlineStr"/>
+    </row>
+    <row r="46" ht="22" customHeight="1">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D045.jpg</t>
+        </is>
+      </c>
+      <c r="B46" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D045</t>
+        </is>
+      </c>
+      <c r="C46" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con militar chino en escritorio, gráfica de Nebivolol, cuadrado rojo y dibujo de mano]</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por la ilustración de un militante socialista chino sentado escribiendo en su escritorio, una gráfica estadística comparativa de variación clínica ("Nebivolol"), un cuadrado de papel rojo intenso, el dibujo esquemático de una mano sujetando un instrumental y un elemento recortado en forma de prenda suspendida. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr"/>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J46" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K46" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L46" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Propaganda china, Cardiología, Los correctores</t>
+        </is>
+      </c>
+      <c r="M46" s="3" t="inlineStr"/>
+    </row>
+    <row r="47" ht="22" customHeight="1">
+      <c r="A47" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D046.jpg</t>
+        </is>
+      </c>
+      <c r="B47" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D046</t>
+        </is>
+      </c>
+      <c r="C47" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D47" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con gasolinera Cepsa, dibujo anatómico de hernia hiatal y satélite en el espacio]</t>
+        </is>
+      </c>
+      <c r="E47" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por una fotografía recortada de una estación de servicio de la marca Cepsa iluminada de noche, un dibujo anatómico impreso del aparato digestivo con rótulos médicos ("Aclaramiento esofágico", "Relajación transitoria", "Hernia hiatal", "Retraso vaciado gástrico") y una fotografía en el espacio exterior de un satélite artificial sobre la curvatura de la Tierra. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F47" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G47" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H47" s="2" t="inlineStr"/>
+      <c r="I47" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J47" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K47" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L47" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Gasolinera Cepsa, Anatomía, Satélite, Los correctores</t>
+        </is>
+      </c>
+      <c r="M47" s="3" t="inlineStr"/>
+    </row>
+    <row r="48" ht="22" customHeight="1">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D047.jpg</t>
+        </is>
+      </c>
+      <c r="B48" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D047</t>
+        </is>
+      </c>
+      <c r="C48" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con arco de tablillas asiáticas escritas, mar, caracola y pintor ante caballete]</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por una estructura en forma de arco o pórtico formada por tablillas de madera impresas con caracteres y caligrafía asiática/japonesa, sobre un fondo fotográfico de paisaje marino, un medallón circular con la silueta de un pintor trabajando ante su caballete y una ilustración en tono azulado de una caracola marina. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr"/>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J48" s="3" t="inlineStr">
+        <is>
+          <t>Collage sobre papel</t>
+        </is>
+      </c>
+      <c r="K48" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L48" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Orientalismo, Caracola, Pintor, Los correctores</t>
+        </is>
+      </c>
+      <c r="M48" s="3" t="inlineStr"/>
+    </row>
+    <row r="49" ht="22" customHeight="1">
+      <c r="A49" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D048.jpg</t>
+        </is>
+      </c>
+      <c r="B49" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-EXPOSICIONES-C010-P001-D048</t>
+        </is>
+      </c>
+      <c r="C49" s="2" t="inlineStr">
+        <is>
+          <t>C010-P001</t>
+        </is>
+      </c>
+      <c r="D49" s="3" t="inlineStr">
+        <is>
+          <t>[Collage de Quico Rivas con media cáscara de huevo rellena, mástil y vela triangular trazada a tinta]</t>
+        </is>
+      </c>
+      <c r="E49" s="3" t="inlineStr">
+        <is>
+          <t>Collage original de Quico Rivas compuesto por un recorte fotográfico de medio huevo cocido relleno (estilo huevo relleno con aceituna), sobre el que el autor ha trazado a tinta negra una línea vertical a modo de mástil coronada por un gran triángulo geométrico transparente que simula la vela de una embarcación. Firmado por el autor como "Q 2000". Formaba parte de la agrupación descrita en la nota manuscrita: "Los correctores, esquema 1f. carpeta El libro rojo para pasar a Galvez Expo. Sev. 09/2018".</t>
+        </is>
+      </c>
+      <c r="F49" s="2" t="inlineStr">
+        <is>
+          <t>2000</t>
+        </is>
+      </c>
+      <c r="G49" s="2" t="inlineStr">
+        <is>
+          <t>EXPOSICIONES</t>
+        </is>
+      </c>
+      <c r="H49" s="2" t="inlineStr"/>
+      <c r="I49" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J49" s="3" t="inlineStr">
+        <is>
+          <t>Collage y tinta sobre papel</t>
+        </is>
+      </c>
+      <c r="K49" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas</t>
+        </is>
+      </c>
+      <c r="L49" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, Collage, Poesía visual, Gastronomía, Los correctores</t>
+        </is>
+      </c>
+      <c r="M49" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M9"/>
+  <autoFilter ref="A1:M49"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Normalización del tesauro de materias (subject) a 14 categorías generales
</commit_message>
<xml_diff>
--- a/Nivel 9 (Documento simple).xlsx
+++ b/Nivel 9 (Documento simple).xlsx
@@ -597,7 +597,7 @@
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Guerra Civil Española, Atarazanas, Recortables, Memoria histórica, Ilustraciones</t>
+          <t>Memoria Histórica y Guerra Civil, Edición y Publicaciones, Objetos y Cultura Material</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr"/>
@@ -656,7 +656,7 @@
       </c>
       <c r="L3" s="3" t="inlineStr">
         <is>
-          <t>Columna Durruti, Milicias del Pueblo, CNT-FAI, Anarquismo, Propaganda de guerra</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Memoria Histórica y Guerra Civil, Propaganda Política e Ideología</t>
         </is>
       </c>
       <c r="M3" s="3" t="inlineStr"/>
@@ -711,7 +711,7 @@
       <c r="K4" s="3" t="inlineStr"/>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>El Refractor, Sellos de caucho, Imprenta, Movimiento libertario, Objetos</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Edición y Publicaciones, Diseño Gráfico y Tipografía</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="L5" s="3" t="inlineStr">
         <is>
-          <t>Sindicato Único, Industrias Químicas, CNT-AIT, Colectivizaciones, Cerillas</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Memoria Histórica y Guerra Civil, Objetos y Cultura Material</t>
         </is>
       </c>
       <c r="M5" s="3" t="inlineStr">
@@ -841,7 +841,7 @@
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Anarquismo individualista, Émile Armand, Pepitas de Calabaza, Libros, Ex-libris</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Edición y Publicaciones, Diseño Gráfico y Tipografía</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
@@ -900,7 +900,7 @@
       <c r="K7" s="3" t="inlineStr"/>
       <c r="L7" s="3" t="inlineStr">
         <is>
-          <t>Abstencionismo, Casas Viejas, Segunda República, Pasquines, Propaganda</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Memoria Histórica y Guerra Civil, Propaganda Política e Ideología</t>
         </is>
       </c>
       <c r="M7" s="3" t="inlineStr">
@@ -963,7 +963,7 @@
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>José Díaz, Partido Comunista de España, Banderines, Simbología política, Guerra Civil Española</t>
+          <t>Memoria Histórica y Guerra Civil, Propaganda Política e Ideología, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
@@ -1026,7 +1026,7 @@
       </c>
       <c r="L9" s="3" t="inlineStr">
         <is>
-          <t>Servicio de Investigación Militar, Banderas, Segunda República, Guiones militares, Guerra Civil Española</t>
+          <t>Memoria Histórica y Guerra Civil, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M9" s="3" t="inlineStr">
@@ -1089,7 +1089,7 @@
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Alfonso Laurencic, Chekas, Guerra Civil Española, Correspondencia</t>
+          <t>Memoria Histórica y Guerra Civil, Arquitectura y Espacio Urbano, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr"/>
@@ -1152,7 +1152,7 @@
       </c>
       <c r="L11" s="3" t="inlineStr">
         <is>
-          <t>CO.IN, Quico Rivas, Grazalema, Comunicados, Manuscritos</t>
+          <t>Crítica de Arte y Comisariado, Correspondencia y Documentación Personal, Artes Plásticas y Visuales, Poesía Visual y Literatura</t>
         </is>
       </c>
       <c r="M11" s="3" t="inlineStr"/>
@@ -1211,7 +1211,7 @@
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>El Refractor, Archivo Refractor, CEDCS, Custodia de documentos</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr"/>
@@ -1266,7 +1266,7 @@
       <c r="K13" s="3" t="inlineStr"/>
       <c r="L13" s="3" t="inlineStr">
         <is>
-          <t>Bocetos, Diseño gráfico, Contracultura, Obra gráfica</t>
+          <t>Diseño Gráfico y Tipografía, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M13" s="3" t="inlineStr"/>
@@ -1325,7 +1325,7 @@
       </c>
       <c r="L14" s="3" t="inlineStr">
         <is>
-          <t>Daniel Zarza, URSS, Alejandro Rossi, Caligrafía, Tarjetas postales</t>
+          <t>Artes Plásticas y Visuales, Poesía Visual y Literatura</t>
         </is>
       </c>
       <c r="M14" s="3" t="inlineStr"/>
@@ -1380,7 +1380,7 @@
       <c r="K15" s="3" t="inlineStr"/>
       <c r="L15" s="3" t="inlineStr">
         <is>
-          <t>Kazimir Malevich, Suprematismo, Collage, Zarza, Z®Z</t>
+          <t>Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M15" s="3" t="inlineStr"/>
@@ -1435,7 +1435,7 @@
       <c r="K16" s="3" t="inlineStr"/>
       <c r="L16" s="3" t="inlineStr">
         <is>
-          <t>Kazimir Malevich, Suprematismo, Collage, Zarza, Z®Z</t>
+          <t>Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M16" s="3" t="inlineStr"/>
@@ -1498,7 +1498,7 @@
       </c>
       <c r="L17" s="3" t="inlineStr">
         <is>
-          <t>El Ojo Atómico, El Refractor, Domingo Negro, Bocángel 59, Carteles</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Diseño Gráfico y Tipografía, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M17" s="3" t="inlineStr"/>
@@ -1557,7 +1557,7 @@
       </c>
       <c r="L18" s="3" t="inlineStr">
         <is>
-          <t>El Refractor, Quico Rivas, SEMEFO, Galería Cruce, ZAT, KAX-1013</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Crítica de Arte y Comisariado, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M18" s="3" t="inlineStr"/>
@@ -1616,7 +1616,7 @@
       </c>
       <c r="L19" s="3" t="inlineStr">
         <is>
-          <t>Fotografía, Rafa Montesinos, Anarquismo, Grafitis</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Fotografía y Registro Audiovisual</t>
         </is>
       </c>
       <c r="M19" s="3" t="inlineStr"/>
@@ -1675,7 +1675,7 @@
       </c>
       <c r="L20" s="3" t="inlineStr">
         <is>
-          <t>Maraviles, Contracultura, Cortes de luz, Comunicados</t>
+          <t>Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M20" s="3" t="inlineStr"/>
@@ -1738,7 +1738,7 @@
       </c>
       <c r="L21" s="3" t="inlineStr">
         <is>
-          <t>Bocángel, Carteles, Anarquismo, Imprenta, Notas manuscritas</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Edición y Publicaciones, Diseño Gráfico y Tipografía</t>
         </is>
       </c>
       <c r="M21" s="3" t="inlineStr"/>
@@ -1801,7 +1801,7 @@
       </c>
       <c r="L22" s="3" t="inlineStr">
         <is>
-          <t>Barcelona, Recortables, Guerra Civil Española, Atarazanas, Dioramas</t>
+          <t>Memoria Histórica y Guerra Civil, Objetos y Cultura Material</t>
         </is>
       </c>
       <c r="M22" s="3" t="inlineStr"/>
@@ -1856,7 +1856,7 @@
       <c r="K23" s="3" t="inlineStr"/>
       <c r="L23" s="3" t="inlineStr">
         <is>
-          <t>Collage, Rafael Zarza, Artes gráficas, Cine, Teatro</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M23" s="3" t="inlineStr"/>
@@ -1915,7 +1915,7 @@
       </c>
       <c r="L24" s="3" t="inlineStr">
         <is>
-          <t>CNT-AIT, Sindicato del Espectáculo, Collage, Anarcosindicato, Diseño gráfico</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Diseño Gráfico y Tipografía, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M24" s="3" t="inlineStr"/>
@@ -1970,7 +1970,7 @@
       <c r="K25" s="3" t="inlineStr"/>
       <c r="L25" s="3" t="inlineStr">
         <is>
-          <t>Ediciones Refractarias, Bocetos, Diseños de logotipo, El Refractor, Rafael Zarza</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Diseño Gráfico y Tipografía, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M25" s="3" t="inlineStr"/>
@@ -2025,7 +2025,7 @@
       <c r="K26" s="3" t="inlineStr"/>
       <c r="L26" s="3" t="inlineStr">
         <is>
-          <t>Ediciones Refractarias, Bocetos, Diseños de logotipo, El Refractor, Rafael Zarza</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Diseño Gráfico y Tipografía, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M26" s="3" t="inlineStr"/>
@@ -2080,7 +2080,7 @@
       <c r="K27" s="3" t="inlineStr"/>
       <c r="L27" s="3" t="inlineStr">
         <is>
-          <t>Ediciones Refractarias, Anarquismo, Logotipos, El Refractor, Rafael Zarza</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Diseño Gráfico y Tipografía, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M27" s="3" t="inlineStr"/>
@@ -2135,7 +2135,7 @@
       <c r="K28" s="3" t="inlineStr"/>
       <c r="L28" s="3" t="inlineStr">
         <is>
-          <t>Ediciones Refractarias, Anarquismo, Logotipos, El Refractor, Rafael Zarza</t>
+          <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Diseño Gráfico y Tipografía, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M28" s="3" t="inlineStr"/>
@@ -2194,7 +2194,7 @@
       </c>
       <c r="L29" s="3" t="inlineStr">
         <is>
-          <t>Josechu Dávila, Papel cebolla, Geometría, Obra pictórica</t>
+          <t>Arquitectura y Espacio Urbano</t>
         </is>
       </c>
       <c r="M29" s="3" t="inlineStr"/>
@@ -2249,7 +2249,7 @@
       <c r="K30" s="3" t="inlineStr"/>
       <c r="L30" s="3" t="inlineStr">
         <is>
-          <t>Las otras galerías, Panóptico de Bentham, Panóptico digital, Design collage, Rafael Zarza</t>
+          <t>Diseño Gráfico y Tipografía, Artes Plásticas y Visuales, Crítica de Arte y Comisariado, Arquitectura y Espacio Urbano</t>
         </is>
       </c>
       <c r="M30" s="3" t="inlineStr"/>
@@ -2308,7 +2308,7 @@
       </c>
       <c r="L31" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Esfera terrestre, Lupa, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Correspondencia y Documentación Personal, Poesía Visual y Literatura</t>
         </is>
       </c>
       <c r="M31" s="3" t="inlineStr"/>
@@ -2367,7 +2367,7 @@
       </c>
       <c r="L32" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Propaganda china, Automóvil clásico, Los correctores</t>
+          <t>Propaganda Política e Ideología, Edición y Publicaciones, Diseño Gráfico y Tipografía, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M32" s="3" t="inlineStr"/>
@@ -2426,7 +2426,7 @@
       </c>
       <c r="L33" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Anatomía, Odontología, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M33" s="3" t="inlineStr"/>
@@ -2485,7 +2485,7 @@
       </c>
       <c r="L34" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Calavera, Gafas de sol, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Correspondencia y Documentación Personal, Poesía Visual y Literatura</t>
         </is>
       </c>
       <c r="M34" s="3" t="inlineStr"/>
@@ -2544,7 +2544,7 @@
       </c>
       <c r="L35" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Automóvil deportivo, Moldes dentales, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M35" s="3" t="inlineStr"/>
@@ -2603,7 +2603,7 @@
       </c>
       <c r="L36" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Diagrama médico, Flor, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M36" s="3" t="inlineStr"/>
@@ -2662,7 +2662,7 @@
       </c>
       <c r="L37" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Cápsula farmacéutica, Boca, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M37" s="3" t="inlineStr"/>
@@ -2721,7 +2721,7 @@
       </c>
       <c r="L38" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Biofarmacia, Ergonomía, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M38" s="3" t="inlineStr"/>
@@ -2780,7 +2780,7 @@
       </c>
       <c r="L39" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Odontología, Instrumental médico, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M39" s="3" t="inlineStr"/>
@@ -2839,7 +2839,7 @@
       </c>
       <c r="L40" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Abstracción, Odontología, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M40" s="3" t="inlineStr"/>
@@ -2898,7 +2898,7 @@
       </c>
       <c r="L41" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Gafas de sol, Anatomía ocular, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M41" s="3" t="inlineStr"/>
@@ -2957,7 +2957,7 @@
       </c>
       <c r="L42" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Propaganda china, Cardiología, Los correctores</t>
+          <t>Memoria Histórica y Guerra Civil, Propaganda Política e Ideología, Edición y Publicaciones, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M42" s="3" t="inlineStr"/>
@@ -3020,7 +3020,7 @@
       </c>
       <c r="L43" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Sevilla, Tráfico, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Arquitectura y Espacio Urbano, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M43" s="3" t="inlineStr"/>
@@ -3079,7 +3079,7 @@
       </c>
       <c r="L44" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Propaganda china, Farmacología, Los correctores</t>
+          <t>Memoria Histórica y Guerra Civil, Propaganda Política e Ideología, Edición y Publicaciones, Diseño Gráfico y Tipografía</t>
         </is>
       </c>
       <c r="M44" s="3" t="inlineStr"/>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="L45" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Propaganda china, Micrografía, Los correctores</t>
+          <t>Memoria Histórica y Guerra Civil, Propaganda Política e Ideología, Edición y Publicaciones, Artes Plásticas y Visuales</t>
         </is>
       </c>
       <c r="M45" s="3" t="inlineStr"/>
@@ -3197,7 +3197,7 @@
       </c>
       <c r="L46" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Propaganda china, Cardiología, Los correctores</t>
+          <t>Propaganda Política e Ideología, Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias</t>
         </is>
       </c>
       <c r="M46" s="3" t="inlineStr"/>
@@ -3256,7 +3256,7 @@
       </c>
       <c r="L47" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Gasolinera Cepsa, Anatomía, Satélite, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Medicina y Ciencias, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M47" s="3" t="inlineStr"/>
@@ -3315,7 +3315,7 @@
       </c>
       <c r="L48" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Orientalismo, Caracola, Pintor, Los correctores</t>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Correspondencia y Documentación Personal, Poesía Visual y Literatura</t>
         </is>
       </c>
       <c r="M48" s="3" t="inlineStr"/>
@@ -3374,7 +3374,7 @@
       </c>
       <c r="L49" s="3" t="inlineStr">
         <is>
-          <t>Quico Rivas, Collage, Poesía visual, Gastronomía, Los correctores</t>
+          <t>Memoria Histórica y Guerra Civil, Edición y Publicaciones, Artes Plásticas y Visuales, Correspondencia y Documentación Personal</t>
         </is>
       </c>
       <c r="M49" s="3" t="inlineStr"/>

</xml_diff>

<commit_message>
Actualizacion de catalogacion Nivel 7 y Nivel 9, optimizaciones de rendimiento y correccion de ubicaciones C128 (D003-D006, D065-D068)
</commit_message>
<xml_diff>
--- a/Nivel 9 (Documento simple).xlsx
+++ b/Nivel 9 (Documento simple).xlsx
@@ -10,7 +10,7 @@
     <sheet name="Nivel 9 (Documento simple)" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nivel 9 (Documento simple)'!$A$1:$M$49</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Nivel 9 (Documento simple)'!$A$1:$M$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -454,7 +454,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M49"/>
+  <dimension ref="A1:M69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -664,17 +664,17 @@
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D003.jpg</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C128-D003.jpg</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D003</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C128-D003</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>C001-P001</t>
+          <t>C128</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -714,26 +714,22 @@
           <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Edición y Publicaciones, Diseño Gráfico y Tipografía</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
-        <is>
-          <t>Ubicacion física no definitiva</t>
-        </is>
-      </c>
+      <c r="M4" s="3" t="inlineStr"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D004.jpg</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C128-D004.jpg</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D004</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C128-D004</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>C001-P001</t>
+          <t>C128</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -777,26 +773,22 @@
           <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Memoria Histórica y Guerra Civil, Objetos y Cultura Material</t>
         </is>
       </c>
-      <c r="M5" s="3" t="inlineStr">
-        <is>
-          <t>Ubicacion física no definitiva</t>
-        </is>
-      </c>
+      <c r="M5" s="3" t="inlineStr"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D005.jpg</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C128-D005.jpg</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C001-P001-D005</t>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C128-D005</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>C001-P001</t>
+          <t>C128</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -844,26 +836,22 @@
           <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Edición y Publicaciones, Diseño Gráfico y Tipografía</t>
         </is>
       </c>
-      <c r="M6" s="3" t="inlineStr">
-        <is>
-          <t>Ubicacion física no definitiva</t>
-        </is>
-      </c>
+      <c r="M6" s="3" t="inlineStr"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D006.jpg</t>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C128-D006.jpg</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D006</t>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C128-D006</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>C001-P001</t>
+          <t>C128</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -903,26 +891,22 @@
           <t>Movimiento Libertario y Anarquismo, Contracultura y Subversión, Memoria Histórica y Guerra Civil, Propaganda Política e Ideología</t>
         </is>
       </c>
-      <c r="M7" s="3" t="inlineStr">
-        <is>
-          <t>Ubicacion física no definitiva</t>
-        </is>
-      </c>
+      <c r="M7" s="3" t="inlineStr"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D007.jpg</t>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C118-P001-D007.jpg</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D007</t>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C118-P001-D007</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>C001-P001</t>
+          <t>C118-P001</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -966,26 +950,22 @@
           <t>Memoria Histórica y Guerra Civil, Propaganda Política e Ideología, Correspondencia y Documentación Personal</t>
         </is>
       </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>Ubicacion física no definitiva</t>
-        </is>
-      </c>
+      <c r="M8" s="3" t="inlineStr"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D008.jpg</t>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C118-P002-D008.jpg</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>ES-CEDCS-ZARZA-MILITANCIA-C001-P001-D008</t>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C118-P002-D008</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>C001-P001</t>
+          <t>C118-P002</t>
         </is>
       </c>
       <c r="D9" s="3" t="inlineStr">
@@ -1029,11 +1009,7 @@
           <t>Memoria Histórica y Guerra Civil, Correspondencia y Documentación Personal</t>
         </is>
       </c>
-      <c r="M9" s="3" t="inlineStr">
-        <is>
-          <t>Ubicacion física no definitiva</t>
-        </is>
-      </c>
+      <c r="M9" s="3" t="inlineStr"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="2" t="inlineStr">
@@ -3379,8 +3355,1192 @@
       </c>
       <c r="M49" s="3" t="inlineStr"/>
     </row>
+    <row r="50" ht="22" customHeight="1">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D049.jpg</t>
+        </is>
+      </c>
+      <c r="B50" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D049</t>
+        </is>
+      </c>
+      <c r="C50" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de la tienda de loza y porcelana La Vajilla en la Calle del Arenal de Madrid]</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía de la fachada de la tienda de loza y porcelana La Vajilla, situada en la calle del Arenal de Madrid, mostrando escaparates con piezas de vajilla, figuras y cristalería, con transeúntes paseando por la acera.</t>
+        </is>
+      </c>
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr"/>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J50" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K50" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L50" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M50" s="3" t="inlineStr"/>
+    </row>
+    <row r="51" ht="22" customHeight="1">
+      <c r="A51" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D050.jpg</t>
+        </is>
+      </c>
+      <c r="B51" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D050</t>
+        </is>
+      </c>
+      <c r="C51" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D51" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de una limpiadora de cristales trabajando en el escaparate de un comercio en Madrid]</t>
+        </is>
+      </c>
+      <c r="E51" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía de una mujer limpiando los cristales del escaparate de un comercio desde el interior, vista a través del cristal reflectante donde se intuye la calle madrileña.</t>
+        </is>
+      </c>
+      <c r="F51" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G51" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H51" s="2" t="inlineStr"/>
+      <c r="I51" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J51" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K51" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L51" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M51" s="3" t="inlineStr"/>
+    </row>
+    <row r="52" ht="22" customHeight="1">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D051.jpg</t>
+        </is>
+      </c>
+      <c r="B52" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D051</t>
+        </is>
+      </c>
+      <c r="C52" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de una mujer y dos niñas vestidas de blanco paseando por la Gran Vía de Madrid]</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Toma posterior de una mujer acompañada de dos niñas con vestidos blancos de ceremonia caminando por la acera de la Gran Vía de Madrid, con transeúntes y la arquitectura urbana de fondo.</t>
+        </is>
+      </c>
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr"/>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J52" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K52" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L52" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M52" s="3" t="inlineStr"/>
+    </row>
+    <row r="53" ht="22" customHeight="1">
+      <c r="A53" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D052.jpg</t>
+        </is>
+      </c>
+      <c r="B53" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D052</t>
+        </is>
+      </c>
+      <c r="C53" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D53" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de la terraza de un café en la Gran Vía de Madrid]</t>
+        </is>
+      </c>
+      <c r="E53" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía de una terraza con mesas vestidas de mantel blanco y sillas de mimbre en la Gran Vía de Madrid, con clientes sentados y peatones transitando, entre ellos un marinero uniformado.</t>
+        </is>
+      </c>
+      <c r="F53" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G53" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H53" s="2" t="inlineStr"/>
+      <c r="I53" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J53" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K53" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L53" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M53" s="3" t="inlineStr"/>
+    </row>
+    <row r="54" ht="22" customHeight="1">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D053.jpg</t>
+        </is>
+      </c>
+      <c r="B54" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D053</t>
+        </is>
+      </c>
+      <c r="C54" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía en silueta de un peatón bajo la marquesina de la Calle de Alcalá en Madrid]</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Composición fotográfica en contraluz mostrando la silueta de un transeúnte caminando bajo una marquesina acristalada en la acera de la Calle de Alcalá, con un carro de tracción animal y el Hotel Suizo al fondo.</t>
+        </is>
+      </c>
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr"/>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J54" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K54" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L54" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales, Arquitectura y Espacio Urbano</t>
+        </is>
+      </c>
+      <c r="M54" s="3" t="inlineStr"/>
+    </row>
+    <row r="55" ht="22" customHeight="1">
+      <c r="A55" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D054.jpg</t>
+        </is>
+      </c>
+      <c r="B55" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D054</t>
+        </is>
+      </c>
+      <c r="C55" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D55" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de militares y peatones en la Plaza de España de Madrid]</t>
+        </is>
+      </c>
+      <c r="E55" s="3" t="inlineStr">
+        <is>
+          <t>Vista urbana de la Plaza de España de Madrid con soldados uniformados y mujeres paseando frente a las oficinas de TWA y el Edificio España de fondo.</t>
+        </is>
+      </c>
+      <c r="F55" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G55" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H55" s="2" t="inlineStr"/>
+      <c r="I55" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J55" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K55" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L55" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales, Arquitectura y Espacio Urbano</t>
+        </is>
+      </c>
+      <c r="M55" s="3" t="inlineStr"/>
+    </row>
+    <row r="56" ht="22" customHeight="1">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D055.jpg</t>
+        </is>
+      </c>
+      <c r="B56" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D055</t>
+        </is>
+      </c>
+      <c r="C56" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de un joven aprendiz descendiendo por una escalinata en sol y sombra]</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Vista cenital de un joven aprendiz con delantal llevando una caja de madera mientras desciende por unas escaleras exteriores iluminadas con sombras diagonales pronunciadas.</t>
+        </is>
+      </c>
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr"/>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J56" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K56" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L56" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M56" s="3" t="inlineStr"/>
+    </row>
+    <row r="57" ht="22" customHeight="1">
+      <c r="A57" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D056.jpg</t>
+        </is>
+      </c>
+      <c r="B57" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D056</t>
+        </is>
+      </c>
+      <c r="C57" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D57" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía nocturna de un autobús de dos pisos frente al Cine Avenida en Madrid]</t>
+        </is>
+      </c>
+      <c r="E57" s="3" t="inlineStr">
+        <is>
+          <t>Vista nocturna de la Gran Vía madrileña con un autobús de dos pisos de la línea 1 estacionado junto al Cine Avenida, decorado con carteles luminosos de la película Pluma al viento.</t>
+        </is>
+      </c>
+      <c r="F57" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G57" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H57" s="2" t="inlineStr"/>
+      <c r="I57" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J57" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K57" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L57" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales, Arquitectura y Espacio Urbano</t>
+        </is>
+      </c>
+      <c r="M57" s="3" t="inlineStr"/>
+    </row>
+    <row r="58" ht="22" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D057.jpg</t>
+        </is>
+      </c>
+      <c r="B58" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D057</t>
+        </is>
+      </c>
+      <c r="C58" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de un automóvil cubierto de nieve en la Gran Vía de Madrid]</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía de un paisaje urbano invernal en Madrid mostrando un automóvil antiguo cubierto por una capa de nieve estacionado en la acera de la Gran Vía.</t>
+        </is>
+      </c>
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr"/>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J58" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K58" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L58" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M58" s="3" t="inlineStr"/>
+    </row>
+    <row r="59" ht="22" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D058.jpg</t>
+        </is>
+      </c>
+      <c r="B59" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D058</t>
+        </is>
+      </c>
+      <c r="C59" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D59" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de una mujer con vestido a rayas caminando por una acera madrileña]</t>
+        </is>
+      </c>
+      <c r="E59" s="3" t="inlineStr">
+        <is>
+          <t>Vista posterior de una mujer vistiendo un elegante vestido acampanado a rayas y zapatos de tacón paseando por una calle de Madrid entre otros transeúntes.</t>
+        </is>
+      </c>
+      <c r="F59" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G59" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H59" s="2" t="inlineStr"/>
+      <c r="I59" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J59" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K59" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L59" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M59" s="3" t="inlineStr"/>
+    </row>
+    <row r="60" ht="22" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D059.jpg</t>
+        </is>
+      </c>
+      <c r="B60" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D059</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D60" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de una mujer caminando bajo el toldo de un comercio en la Gran Vía de Madrid]</t>
+        </is>
+      </c>
+      <c r="E60" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía urbana con un contraluz acentuado mostrando a una mujer vestida con traje claro caminando hacia la cámara en la acera de la Gran Vía, proyectando una marcada sombra.</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H60" s="2" t="inlineStr"/>
+      <c r="I60" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J60" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K60" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L60" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M60" s="3" t="inlineStr"/>
+    </row>
+    <row r="61" ht="22" customHeight="1">
+      <c r="A61" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D060.jpg</t>
+        </is>
+      </c>
+      <c r="B61" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D060</t>
+        </is>
+      </c>
+      <c r="C61" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D61" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de un joven vendedor ambulante con cesto de mimbre frente al Edificio España de Madrid]</t>
+        </is>
+      </c>
+      <c r="E61" s="3" t="inlineStr">
+        <is>
+          <t>Retrato de plano medio de un joven con boina sosteniendo un cesto de mimbre cargado de figuras pequeñas, con los rascacielos de la Plaza de España de Madrid al fondo.</t>
+        </is>
+      </c>
+      <c r="F61" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G61" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H61" s="2" t="inlineStr"/>
+      <c r="I61" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J61" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K61" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L61" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M61" s="3" t="inlineStr"/>
+    </row>
+    <row r="62" ht="22" customHeight="1">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D061.jpg</t>
+        </is>
+      </c>
+      <c r="B62" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D061</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D62" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía de un hombre haciendo pompas de jabón en la Gran Vía de Madrid]</t>
+        </is>
+      </c>
+      <c r="E62" s="3" t="inlineStr">
+        <is>
+          <t>Toma de perfil de un hombre haciendo pompas de jabón en la vía pública ante la mirada curiosa de varios transeúntes con la arquitectura urbana madrileña de fondo.</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H62" s="2" t="inlineStr"/>
+      <c r="I62" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J62" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K62" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L62" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M62" s="3" t="inlineStr"/>
+    </row>
+    <row r="63" ht="22" customHeight="1">
+      <c r="A63" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D062.jpg</t>
+        </is>
+      </c>
+      <c r="B63" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D062</t>
+        </is>
+      </c>
+      <c r="C63" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D63" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía del templete de acceso al Metro en la Red de San Luis de Madrid]</t>
+        </is>
+      </c>
+      <c r="E63" s="3" t="inlineStr">
+        <is>
+          <t>Vista exterior del templete monumental del Metro diseñado por el arquitecto Antonio Palacios en la Red de San Luis (Gran Vía), con viajeros y transeúntes rodeando la estructura.</t>
+        </is>
+      </c>
+      <c r="F63" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G63" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H63" s="2" t="inlineStr"/>
+      <c r="I63" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J63" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K63" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L63" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales, Arquitectura y Espacio Urbano</t>
+        </is>
+      </c>
+      <c r="M63" s="3" t="inlineStr"/>
+    </row>
+    <row r="64" ht="22" customHeight="1">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D063.jpg</t>
+        </is>
+      </c>
+      <c r="B64" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D063</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D64" s="3" t="inlineStr">
+        <is>
+          <t>[Fotografía nocturna del establecimiento de material fotográfico Boyvi en la Gran Vía de Madrid]</t>
+        </is>
+      </c>
+      <c r="E64" s="3" t="inlineStr">
+        <is>
+          <t>Vista nocturna del escaparate iluminado y luminosos del establecimiento de material fotográfico Boyvi y la tienda España en la Gran Vía madrileña, con la silueta de un viandante en primer plano.</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H64" s="2" t="inlineStr"/>
+      <c r="I64" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J64" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K64" s="3" t="inlineStr">
+        <is>
+          <t>Francesc Català-Roca</t>
+        </is>
+      </c>
+      <c r="L64" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales, Arquitectura y Espacio Urbano</t>
+        </is>
+      </c>
+      <c r="M64" s="3" t="inlineStr"/>
+    </row>
+    <row r="65" ht="22" customHeight="1">
+      <c r="A65" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D064.jpg</t>
+        </is>
+      </c>
+      <c r="B65" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P002-D064</t>
+        </is>
+      </c>
+      <c r="C65" s="2" t="inlineStr">
+        <is>
+          <t>C038-P002</t>
+        </is>
+      </c>
+      <c r="D65" s="3" t="inlineStr">
+        <is>
+          <t>[Retrato fotográfico de la vedette Rosario por el estudio Ibáñez]</t>
+        </is>
+      </c>
+      <c r="E65" s="3" t="inlineStr">
+        <is>
+          <t>Retrato de estudio en blanco y negro de la vedette Rosario recostada de lado en traje de espectáculo junto a una mantilla de encaje suspendida. Presenta firma de Ibáñez en el ángulo superior derecho del anverso. En el dorso incluye sello tampón en tinta morada del estudio fotográfico Ibáñez («PROHIBIDA LA REPRODUCCIÓN DE ESTA FOTO SI NO CONSTA EL NOMBRE DE SU AUTOR. Ibáñez. Avda. José Antonio, 70-1º izqd. MADRID»), anotación manuscrita «Rosario» e indicativo numérico «145». Pertenece a una serie de fotografías de vedetes que en ocasiones presentan sello de estudio en el dorso y en otras carecen de él.</t>
+        </is>
+      </c>
+      <c r="F65" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G65" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H65" s="2" t="inlineStr"/>
+      <c r="I65" s="2" t="inlineStr">
+        <is>
+          <t>Still Image</t>
+        </is>
+      </c>
+      <c r="J65" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía en blanco y negro sobre papel</t>
+        </is>
+      </c>
+      <c r="K65" s="3" t="inlineStr">
+        <is>
+          <t>Estudio Ibáñez</t>
+        </is>
+      </c>
+      <c r="L65" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Artes Plásticas y Visuales</t>
+        </is>
+      </c>
+      <c r="M65" s="3" t="inlineStr"/>
+    </row>
+    <row r="66" ht="22" customHeight="1">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P001-D065.jpg</t>
+        </is>
+      </c>
+      <c r="B66" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-AUDIOVISUAL-C038-P001-D065</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>C038-P001</t>
+        </is>
+      </c>
+      <c r="D66" s="3" t="inlineStr">
+        <is>
+          <t>[Contenedor metálico de conservación de la película documental La generación del 27]</t>
+        </is>
+      </c>
+      <c r="E66" s="3" t="inlineStr">
+        <is>
+          <t>Contenedor metálico circular de conservación para película cinematográfica, con etiqueta impresa del laboratorio cinematográfico Cinematiraje Riera S.A. («General Díaz Porlier, 101... MADRID-6»). Incluye título mecanografiado «LA GENERACION DEL 27» e indicativo «1 COPIA». La unidad conserva en su interior una copia de la película cinematográfica documental del mismo título.</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>AUDIOVISUAL</t>
+        </is>
+      </c>
+      <c r="H66" s="2" t="inlineStr">
+        <is>
+          <t>Madrid, Calle General Díaz Porlier</t>
+        </is>
+      </c>
+      <c r="I66" s="2" t="inlineStr">
+        <is>
+          <t>Physical Object</t>
+        </is>
+      </c>
+      <c r="J66" s="3" t="inlineStr">
+        <is>
+          <t>Contenedor metálico circular con etiqueta de papel impreso</t>
+        </is>
+      </c>
+      <c r="K66" s="3" t="inlineStr">
+        <is>
+          <t>Cinematiraje Riera S.A.</t>
+        </is>
+      </c>
+      <c r="L66" s="3" t="inlineStr">
+        <is>
+          <t>Fotografía y Registro Audiovisual, Objetos y Cultura Material, Edición y Publicaciones</t>
+        </is>
+      </c>
+      <c r="M66" s="3" t="inlineStr"/>
+    </row>
+    <row r="67" ht="22" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C029-P003-D066.jpg</t>
+        </is>
+      </c>
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PUBLICACIONES-C029-P003-D066</t>
+        </is>
+      </c>
+      <c r="C67" s="2" t="inlineStr">
+        <is>
+          <t>C029-P003</t>
+        </is>
+      </c>
+      <c r="D67" s="3" t="inlineStr">
+        <is>
+          <t>THE DYNAMITE</t>
+        </is>
+      </c>
+      <c r="E67" s="3" t="inlineStr">
+        <is>
+          <t>Fanzine memorial titulado THE DYNAMITE (subtitulado ZERO), elaborado artesanalmente a mano por Rafael Zarza y dedicado a Rafael Feo en mayo de 2006. Objeto documental encuadernado que comprende collages, notas autógrafas e ilustraciones originales, presentando en cubierta la composición dibujada «Proyecto para monumento sito Plaza de Castilla».</t>
+        </is>
+      </c>
+      <c r="F67" s="2" t="inlineStr">
+        <is>
+          <t>2006-05</t>
+        </is>
+      </c>
+      <c r="G67" s="2" t="inlineStr">
+        <is>
+          <t>PUBLICACIONES</t>
+        </is>
+      </c>
+      <c r="H67" s="2" t="inlineStr">
+        <is>
+          <t>Madrid, Plaza de Castilla</t>
+        </is>
+      </c>
+      <c r="I67" s="2" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="J67" s="3" t="inlineStr">
+        <is>
+          <t>Fanzine artesanal encuadernado a mano con collages, dibujos y notas manuscritas</t>
+        </is>
+      </c>
+      <c r="K67" s="3" t="inlineStr">
+        <is>
+          <t>Rafael Feo</t>
+        </is>
+      </c>
+      <c r="L67" s="3" t="inlineStr">
+        <is>
+          <t>Edición y Publicaciones, Artes Plásticas y Visuales, Poesía Visual y Literatura, Contracultura y Subversión</t>
+        </is>
+      </c>
+      <c r="M67" s="3" t="inlineStr"/>
+    </row>
+    <row r="68" ht="22" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C127-P001-D067.jpg</t>
+        </is>
+      </c>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-MILITANCIA-C127-P001-D067</t>
+        </is>
+      </c>
+      <c r="C68" s="2" t="inlineStr">
+        <is>
+          <t>C127-P001</t>
+        </is>
+      </c>
+      <c r="D68" s="3" t="inlineStr">
+        <is>
+          <t>[Maqueta a escala de vehículo blindado de la CNT-FAI y UGT de la Guerra Civil española]</t>
+        </is>
+      </c>
+      <c r="E68" s="3" t="inlineStr">
+        <is>
+          <t>Maqueta a escala realizada artesanalmente de un vehículo blindado («tiznao») utilizado por la CNT-FAI y la UGT durante la Guerra Civil española. Presenta inscripciones rotuladas en los laterales «F.A.I. C.N.T.», «U.G.T.» y consignas en el frontal como «VIVA LOS MINEROS DE NERVA» y «POR LOS 300 JUDAS».</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>MILITANCIA</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr"/>
+      <c r="I68" s="2" t="inlineStr">
+        <is>
+          <t>Physical Object</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Maqueta a escala tridimensional modelada y pintada sobre chasis de plástico y madera</t>
+        </is>
+      </c>
+      <c r="K68" s="3" t="inlineStr"/>
+      <c r="L68" s="3" t="inlineStr">
+        <is>
+          <t>Objetos y Cultura Material, Memoria Histórica y Guerra Civil, Movimiento Libertario y Anarquismo, Propaganda Política e Ideología</t>
+        </is>
+      </c>
+      <c r="M68" s="3" t="inlineStr"/>
+    </row>
+    <row r="69" ht="22" customHeight="1">
+      <c r="A69" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C127-P001-D068.jpg</t>
+        </is>
+      </c>
+      <c r="B69" s="2" t="inlineStr">
+        <is>
+          <t>ES-CEDCS-ZARZA-PERSONAL-C127-P001-D068</t>
+        </is>
+      </c>
+      <c r="C69" s="2" t="inlineStr">
+        <is>
+          <t>C127-P001</t>
+        </is>
+      </c>
+      <c r="D69" s="3" t="inlineStr">
+        <is>
+          <t>[Bolsa de cuero etiquetada Ojo sanguinolento de Quico Rivas, conservado por María Soberón]</t>
+        </is>
+      </c>
+      <c r="E69" s="3" t="inlineStr">
+        <is>
+          <t>Bolsa de cuero de conservación con etiqueta manuscrita en cartón («OJO SANGUINOLENTO DE QUICO RIVAS (CONSERVADO POR MARÍA SOBERÓN)»), que contiene en su interior una bolsita hermética con una recreación de plástico de un ojo ensangrentado.</t>
+        </is>
+      </c>
+      <c r="F69" s="2" t="inlineStr">
+        <is>
+          <t>[s.f.]</t>
+        </is>
+      </c>
+      <c r="G69" s="2" t="inlineStr">
+        <is>
+          <t>PERSONAL</t>
+        </is>
+      </c>
+      <c r="H69" s="2" t="inlineStr"/>
+      <c r="I69" s="2" t="inlineStr">
+        <is>
+          <t>Physical Object</t>
+        </is>
+      </c>
+      <c r="J69" s="3" t="inlineStr">
+        <is>
+          <t>Bolsa de cuero con etiqueta de cartón manuscrita y bolsa plástica con objeto de plástico</t>
+        </is>
+      </c>
+      <c r="K69" s="3" t="inlineStr">
+        <is>
+          <t>Quico Rivas, María Soberón</t>
+        </is>
+      </c>
+      <c r="L69" s="3" t="inlineStr">
+        <is>
+          <t>Objetos y Cultura Material, Contracultura y Subversión, Crítica de Arte y Comisariado, Correspondencia y Documentación Personal</t>
+        </is>
+      </c>
+      <c r="M69" s="3" t="inlineStr"/>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:M49"/>
+  <autoFilter ref="A1:M69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>